<commit_message>
Pulling y actualizacion del time
</commit_message>
<xml_diff>
--- a/data_mock/Datos.xlsx
+++ b/data_mock/Datos.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18345" windowHeight="10860" activeTab="3"/>
+    <workbookView windowWidth="12285" windowHeight="9360" tabRatio="825" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="pH" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="73">
   <si>
     <t>ID</t>
   </si>
@@ -179,6 +179,12 @@
     <t>M-029</t>
   </si>
   <si>
+    <t>M-009</t>
+  </si>
+  <si>
+    <t>0.01 mg/L</t>
+  </si>
+  <si>
     <t>&lt;1 UFC/mL</t>
   </si>
   <si>
@@ -203,9 +209,6 @@
     <t>M-003</t>
   </si>
   <si>
-    <t>0.01 mg/L</t>
-  </si>
-  <si>
     <t>M-010</t>
   </si>
   <si>
@@ -221,9 +224,6 @@
     <t>M-038</t>
   </si>
   <si>
-    <t>M-009</t>
-  </si>
-  <si>
     <t>3.5 NTU</t>
   </si>
   <si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>M-041</t>
+  </si>
+  <si>
+    <t>451 µS/cm</t>
   </si>
   <si>
     <t>120 mg/L</t>
@@ -264,14 +267,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -727,148 +723,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1580,7 +1576,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
         <v>31</v>
@@ -1597,7 +1593,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -1614,7 +1610,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
@@ -1625,13 +1621,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -1648,7 +1644,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -1665,7 +1661,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -1682,7 +1678,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -1699,7 +1695,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D9" t="s">
         <v>14</v>
@@ -1716,7 +1712,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D10" t="s">
         <v>8</v>
@@ -1733,7 +1729,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -1750,7 +1746,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D12" t="s">
         <v>8</v>
@@ -1767,7 +1763,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -1784,7 +1780,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1801,7 +1797,7 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -1819,7 +1815,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2109,6 +2105,23 @@
       </c>
       <c r="E17" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2148,7 +2161,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -2165,7 +2178,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
         <v>31</v>
@@ -2182,7 +2195,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
@@ -2199,7 +2212,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
@@ -2210,13 +2223,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
         <v>14</v>
@@ -2233,7 +2246,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -2250,7 +2263,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -2267,7 +2280,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -2284,7 +2297,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s">
         <v>8</v>
@@ -2301,7 +2314,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -2312,13 +2325,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
         <v>49</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" t="s">
-        <v>47</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
@@ -2335,7 +2348,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -2352,7 +2365,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
         <v>21</v>
@@ -2369,7 +2382,7 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -2380,13 +2393,13 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
         <v>8</v>
@@ -2403,7 +2416,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
         <v>8</v>
@@ -2414,13 +2427,13 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
         <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
         <v>21</v>
@@ -2431,19 +2444,19 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
         <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D19" t="s">
         <v>14</v>
       </c>
       <c r="E19" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2480,13 +2493,13 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -2503,7 +2516,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
         <v>31</v>
@@ -2520,7 +2533,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
         <v>31</v>
@@ -2537,7 +2550,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2548,13 +2561,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
         <v>14</v>
@@ -2565,13 +2578,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
         <v>21</v>
@@ -2582,13 +2595,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
         <v>31</v>
@@ -2605,7 +2618,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -2616,13 +2629,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -2633,13 +2646,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -2656,7 +2669,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -2667,13 +2680,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s">
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -2690,7 +2703,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
         <v>21</v>
@@ -2707,7 +2720,7 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
         <v>14</v>
@@ -2718,13 +2731,13 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D16" t="s">
         <v>21</v>
@@ -2735,13 +2748,13 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B17" t="s">
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
         <v>8</v>
@@ -2758,7 +2771,7 @@
         <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D18" t="s">
         <v>31</v>
@@ -2769,13 +2782,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="B19" t="s">
         <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D19" t="s">
         <v>31</v>
@@ -2832,7 +2845,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -2934,7 +2947,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
@@ -2975,7 +2988,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3048,7 +3061,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -3065,7 +3078,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -3082,7 +3095,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -3231,6 +3244,23 @@
       </c>
       <c r="E15" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -3270,7 +3300,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
         <v>21</v>
@@ -3287,7 +3317,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
         <v>21</v>
@@ -3304,7 +3334,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -3321,7 +3351,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
@@ -3338,7 +3368,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D6" t="s">
         <v>14</v>
@@ -3355,7 +3385,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
@@ -3372,7 +3402,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -3383,13 +3413,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
@@ -3406,7 +3436,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -3423,7 +3453,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -3440,7 +3470,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -3457,7 +3487,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D13" t="s">
         <v>14</v>
@@ -3474,7 +3504,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -3514,13 +3544,13 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -3537,7 +3567,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
@@ -3548,13 +3578,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
@@ -3565,13 +3595,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>68</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>67</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -3582,13 +3612,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -3605,7 +3635,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -3622,7 +3652,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -3639,7 +3669,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -3650,13 +3680,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -3673,7 +3703,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D11" t="s">
         <v>31</v>
@@ -3684,13 +3714,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
         <v>31</v>
@@ -3707,7 +3737,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -3724,7 +3754,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
         <v>21</v>
@@ -3770,7 +3800,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
         <v>14</v>
@@ -3787,7 +3817,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
         <v>31</v>
@@ -3798,13 +3828,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
@@ -3821,7 +3851,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
@@ -3838,7 +3868,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -3849,13 +3879,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -3866,13 +3896,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -3889,7 +3919,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -3906,7 +3936,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D10" t="s">
         <v>8</v>
@@ -3917,13 +3947,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
         <v>70</v>
-      </c>
-      <c r="B11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" t="s">
-        <v>69</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -3940,7 +3970,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
@@ -3957,7 +3987,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -3974,7 +4004,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D14" t="s">
         <v>31</v>
@@ -3985,13 +4015,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D15" t="s">
         <v>21</v>
@@ -4002,13 +4032,13 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D16" t="s">
         <v>21</v>
@@ -4025,7 +4055,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D17" t="s">
         <v>21</v>

</xml_diff>